<commit_message>
Fiets: gemeten maten (driehoek 46/38/56, stuur binnen 37, 26c, zadelpen 22 cm)
Spreadsheet en masterdocument bijgewerkt; Past? rekent nu met de echte maten.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012qzTUWQo3DsZWfsezFkVX4
</commit_message>
<xml_diff>
--- a/bikepacking_uitrusting.xlsx
+++ b/bikepacking_uitrusting.xlsx
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="192">
   <si>
     <t xml:space="preserve">Bikepacking-uitrusting voor mijn Giant Defy Composite 1 (2012, maat M/L)</t>
   </si>
@@ -173,30 +173,33 @@
     <t xml:space="preserve">Vrije lengte onder de bovenbuis</t>
   </si>
   <si>
-    <t xml:space="preserve">nog meten (schatting 45-50)</t>
+    <t xml:space="preserve">gemeten door eigenaar (driehoek binnen 46 / 38 / 56)</t>
   </si>
   <si>
     <t xml:space="preserve">Langs de onderkant van de bovenbuis, van waar de balhoofdbuis begint tot waar de zitbuis begint. Bepaalt de maximale lengte van een frametas.</t>
   </si>
   <si>
-    <t xml:space="preserve">bidon_ruimte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ruimte bidon (zitbuis) tot bovenbuis</t>
+    <t xml:space="preserve">zitbuis_vrij</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vrije lengte langs de zitbuis (binnen driehoek)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gemeten door eigenaar; geen bidon op de zitbuis (wel boutgaten)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Er zit nu geen bidonhouder op de zitbuis, dus een frametas mag zo hoog als de driehoek toelaat. De onderbuis (binnen 56 cm) heeft wel een bidon.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zadel_band</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ruimte zadelrails tot achterband</t>
   </si>
   <si>
     <t xml:space="preserve">nog meten</t>
   </si>
   <si>
-    <t xml:space="preserve">Met een bidon in de houder: van de dop tot de onderkant van de bovenbuis. Hoe hoog een frametas mag zijn zonder dat de bidon klem zit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zadel_band</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ruimte zadelrails tot achterband</t>
-  </si>
-  <si>
     <t xml:space="preserve">Zadel op rijhoogte: van de zadelrails recht omlaag tot de bovenkant van de achterband. Zadeltassen noemen een minimum (bv. Topeak BackLoader ≥ 9 cm tussen tas en band).</t>
   </si>
   <si>
@@ -206,9 +209,24 @@
     <t xml:space="preserve">Zichtbare zadelpen</t>
   </si>
   <si>
+    <t xml:space="preserve">eerder gemeten door eigenaar</t>
+  </si>
+  <si>
     <t xml:space="preserve">Van de zadelklem op het frame tot de onderkant van de zadelrails. Zadeltassen klemmen hier met een band om de pen (Ortlieb Seat-Pack 11 L: ca. 6 cm).</t>
   </si>
   <si>
+    <t xml:space="preserve">stuur_binnen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stuur binnenmaat (tussen de drops)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gemeten door eigenaar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Een stuurrol of -tas moet hier tussen passen. (Fabrieksmaat van het stuur: Giant Connect SL 42 cm hart op hart.)</t>
+  </si>
+  <si>
     <t xml:space="preserve">stuur_breed</t>
   </si>
   <si>
@@ -299,7 +317,7 @@
     <t xml:space="preserve">waarschijnlijk (47 cm is aan de lange kant)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lichtste frametas in de lijst; waterdicht (IPX6). Lengte is precies het grensgebied — eerst meten.</t>
+    <t xml:space="preserve">Lichtste frametas in de lijst; waterdicht (IPX6). 47 cm is 1 cm langer dan de gemeten 46 cm; met klittenband soms toch te passen, maar niet zeker.</t>
   </si>
   <si>
     <t xml:space="preserve">decathlon.ie, 10-10-2026</t>
@@ -416,7 +434,7 @@
     <t xml:space="preserve">in het zadelharnas hieronder</t>
   </si>
   <si>
-    <t xml:space="preserve">afhankelijk van ruimte zadel-band</t>
+    <t xml:space="preserve">waarschijnlijk: 22 cm zadelpen zichtbaar (ruimte zadel-band nog meten)</t>
   </si>
   <si>
     <t xml:space="preserve">Heeft het zadelharnas (ref. 8579468) nodig; samen ca. €80. Gewicht niet gevonden.</t>
@@ -521,7 +539,7 @@
     <t xml:space="preserve">om het stuur</t>
   </si>
   <si>
-    <t xml:space="preserve">40 cm breed op een 42 cm stuur: krap maar gangbaar</t>
+    <t xml:space="preserve">40 cm breed: te breed voor 37 cm tussen de drops</t>
   </si>
   <si>
     <t xml:space="preserve">Zwaar (492 g). Overweeg de drybag met twee spanbanden in plaats van dit harnas.</t>
@@ -539,7 +557,7 @@
     <t xml:space="preserve">eigen bevestiging, ook carbon stuur</t>
   </si>
   <si>
-    <t xml:space="preserve">de 9 L is de versie voor racesturen</t>
+    <t xml:space="preserve">de 9 L is de versie voor racesturen, maar 40 cm breed</t>
   </si>
   <si>
     <t xml:space="preserve">Waterdicht. UK-prijs £126 (aanbieding); europrijs niet gevonden. Duur voor wat het is.</t>
@@ -852,11 +870,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1371,7 +1389,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -1405,7 +1423,9 @@
       <c r="B2" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="6"/>
+      <c r="C2" s="6" t="n">
+        <v>46</v>
+      </c>
       <c r="D2" s="5" t="s">
         <v>25</v>
       </c>
@@ -1413,14 +1433,16 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
         <v>27</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="6"/>
+      <c r="C3" s="6" t="n">
+        <v>38</v>
+      </c>
       <c r="D3" s="5" t="s">
         <v>29</v>
       </c>
@@ -1435,64 +1457,83 @@
       <c r="B4" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="6"/>
+      <c r="C4" s="7"/>
       <c r="D4" s="5" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" s="6"/>
+        <v>36</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>22</v>
+      </c>
       <c r="D5" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C6" s="7" t="n">
+      <c r="D6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="C7" s="6"/>
       <c r="D7" s="5" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
-        <v>44</v>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="7"/>
+      <c r="D8" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1532,69 +1573,69 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="K1" s="9" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="M1" s="9" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="N1" s="9" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="O1" s="9" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="P1" s="9" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="Q1" s="9" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="C2" s="10" t="n">
         <v>3</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="E2" s="10" t="n">
         <v>150</v>
@@ -1611,7 +1652,7 @@
         <v>25</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J2" s="10" t="n">
         <v>47</v>
@@ -1621,28 +1662,28 @@
       </c>
       <c r="L2" s="5" t="str">
         <f aca="false">IF(OR(J2="",K2=""),M2,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K2,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M2,IF(J2&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K2,'Mijn fiets'!$A:$A,0)),"past","past niet")),M2))</f>
-        <v>nog meten: waarschijnlijk (47 cm is aan de lange kant)</v>
+        <v>past niet</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="P2" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q2" s="6"/>
+        <v>75</v>
+      </c>
+      <c r="Q2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C3" s="10" t="n">
         <v>3.5</v>
@@ -1661,7 +1702,7 @@
         <v>14.2828571428571</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
@@ -1670,31 +1711,31 @@
         <v>afmetingen niet gevonden — nakijken</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="P3" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q3" s="6"/>
+        <v>80</v>
+      </c>
+      <c r="Q3" s="7"/>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="C4" s="10" t="n">
         <v>3</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="E4" s="10" t="n">
         <v>169</v>
@@ -1709,7 +1750,7 @@
         <v/>
       </c>
       <c r="I4" s="5" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="J4" s="10" t="n">
         <v>37.5</v>
@@ -1719,32 +1760,32 @@
       </c>
       <c r="L4" s="5" t="str">
         <f aca="false">IF(OR(J4="",K4=""),M4,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K4,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M4,IF(J4&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K4,'Mijn fiets'!$A:$A,0)),"past","past niet")),M4))</f>
-        <v>nog meten: past</v>
+        <v>past</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="O4" s="5"/>
       <c r="P4" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q4" s="6"/>
+        <v>86</v>
+      </c>
+      <c r="Q4" s="7"/>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C5" s="10" t="n">
         <v>4.5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="E5" s="10" t="n">
         <v>195</v>
@@ -1759,7 +1800,7 @@
         <v/>
       </c>
       <c r="I5" s="5" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>46</v>
@@ -1769,32 +1810,32 @@
       </c>
       <c r="L5" s="5" t="str">
         <f aca="false">IF(OR(J5="",K5=""),M5,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K5,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M5,IF(J5&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K5,'Mijn fiets'!$A:$A,0)),"past","past niet")),M5))</f>
-        <v>nog meten: waarschijnlijk</v>
+        <v>past</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="O5" s="5"/>
       <c r="P5" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q5" s="6"/>
-    </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>91</v>
+      </c>
+      <c r="Q5" s="7"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="C6" s="10" t="n">
         <v>6</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="E6" s="10" t="n">
         <v>337</v>
@@ -1809,7 +1850,7 @@
         <v/>
       </c>
       <c r="I6" s="5" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>54.5</v>
@@ -1819,32 +1860,32 @@
       </c>
       <c r="L6" s="5" t="str">
         <f aca="false">IF(OR(J6="",K6=""),M6,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K6,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M6,IF(J6&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K6,'Mijn fiets'!$A:$A,0)),"past","past niet")),M6))</f>
-        <v>nog meten: waarschijnlijk te lang</v>
+        <v>past niet</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="O6" s="5"/>
       <c r="P6" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q6" s="6"/>
+        <v>86</v>
+      </c>
+      <c r="Q6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C7" s="10" t="n">
         <v>2.4</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="13"/>
@@ -1857,7 +1898,7 @@
         <v/>
       </c>
       <c r="I7" s="5" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>29</v>
@@ -1867,32 +1908,32 @@
       </c>
       <c r="L7" s="5" t="str">
         <f aca="false">IF(OR(J7="",K7=""),M7,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K7,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M7,IF(J7&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K7,'Mijn fiets'!$A:$A,0)),"past","past niet")),M7))</f>
-        <v>nog meten: past</v>
+        <v>past</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="O7" s="5"/>
       <c r="P7" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q7" s="6"/>
+        <v>99</v>
+      </c>
+      <c r="Q7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C8" s="10" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="13"/>
@@ -1905,7 +1946,7 @@
         <v/>
       </c>
       <c r="I8" s="5" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>42</v>
@@ -1915,32 +1956,32 @@
       </c>
       <c r="L8" s="5" t="str">
         <f aca="false">IF(OR(J8="",K8=""),M8,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K8,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M8,IF(J8&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K8,'Mijn fiets'!$A:$A,0)),"past","past niet")),M8))</f>
-        <v>nog meten: waarschijnlijk</v>
+        <v>past</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="N8" s="5" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="O8" s="5"/>
       <c r="P8" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q8" s="6"/>
+        <v>103</v>
+      </c>
+      <c r="Q8" s="7"/>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C9" s="10" t="n">
         <v>4</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E9" s="10" t="n">
         <v>200</v>
@@ -1955,7 +1996,7 @@
         <v/>
       </c>
       <c r="I9" s="5" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>50</v>
@@ -1965,26 +2006,26 @@
       </c>
       <c r="L9" s="5" t="str">
         <f aca="false">IF(OR(J9="",K9=""),M9,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K9,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M9,IF(J9&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K9,'Mijn fiets'!$A:$A,0)),"past","past niet")),M9))</f>
-        <v>nog meten: grensgeval — eerst meten</v>
+        <v>past niet</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="N9" s="5" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="O9" s="5"/>
       <c r="P9" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="Q9" s="6"/>
-    </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>108</v>
+      </c>
+      <c r="Q9" s="7"/>
+    </row>
+    <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>15</v>
@@ -2003,7 +2044,7 @@
         <v>1.4</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="J10" s="5"/>
       <c r="K10" s="5" t="s">
@@ -2011,28 +2052,28 @@
       </c>
       <c r="L10" s="5" t="str">
         <f aca="false">IF(OR(J10="",K10=""),M10,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K10,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M10,IF(J10&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K10,'Mijn fiets'!$A:$A,0)),"past","past niet")),M10))</f>
-        <v>afhankelijk van ruimte zadel-band</v>
+        <v>waarschijnlijk: 22 cm zadelpen zichtbaar (ruimte zadel-band nog meten)</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="P10" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="Q10" s="6"/>
-    </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>114</v>
+      </c>
+      <c r="Q10" s="7"/>
+    </row>
+    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
@@ -2049,7 +2090,7 @@
         <v/>
       </c>
       <c r="I11" s="5" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="J11" s="5"/>
       <c r="K11" s="5" t="s">
@@ -2057,28 +2098,28 @@
       </c>
       <c r="L11" s="5" t="str">
         <f aca="false">IF(OR(J11="",K11=""),M11,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K11,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M11,IF(J11&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K11,'Mijn fiets'!$A:$A,0)),"past","past niet")),M11))</f>
-        <v>afhankelijk van ruimte zadel-band</v>
+        <v>waarschijnlijk: 22 cm zadelpen zichtbaar (ruimte zadel-band nog meten)</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="N11" s="5" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="O11" s="5" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="P11" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="Q11" s="6"/>
+        <v>119</v>
+      </c>
+      <c r="Q11" s="7"/>
     </row>
     <row r="12" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="C12" s="10" t="n">
         <v>6</v>
@@ -2099,7 +2140,7 @@
         <v>7.99333333333333</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="J12" s="5"/>
       <c r="K12" s="5" t="s">
@@ -2107,28 +2148,28 @@
       </c>
       <c r="L12" s="5" t="str">
         <f aca="false">IF(OR(J12="",K12=""),M12,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K12,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M12,IF(J12&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K12,'Mijn fiets'!$A:$A,0)),"past","past niet")),M12))</f>
-        <v>afhankelijk van ruimte zadel-band</v>
+        <v>waarschijnlijk: 22 cm zadelpen zichtbaar (ruimte zadel-band nog meten)</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="N12" s="5" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="O12" s="5" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="P12" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="Q12" s="6"/>
-    </row>
-    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>123</v>
+      </c>
+      <c r="Q12" s="7"/>
+    </row>
+    <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C13" s="10" t="n">
         <v>10</v>
@@ -2149,7 +2190,7 @@
         <v>5.49</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="J13" s="5"/>
       <c r="K13" s="5" t="s">
@@ -2157,28 +2198,28 @@
       </c>
       <c r="L13" s="5" t="str">
         <f aca="false">IF(OR(J13="",K13=""),M13,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K13,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M13,IF(J13&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K13,'Mijn fiets'!$A:$A,0)),"past","past niet")),M13))</f>
-        <v>afhankelijk van ruimte zadel-band</v>
+        <v>waarschijnlijk: 22 cm zadelpen zichtbaar (ruimte zadel-band nog meten)</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="N13" s="5" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="O13" s="5" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="P13" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="Q13" s="6"/>
+        <v>127</v>
+      </c>
+      <c r="Q13" s="7"/>
     </row>
     <row r="14" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C14" s="10" t="n">
         <v>11</v>
@@ -2199,38 +2240,38 @@
         <v>9</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>6</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L14" s="5" t="str">
         <f aca="false">IF(OR(J14="",K14=""),M14,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K14,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M14,IF(J14&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K14,'Mijn fiets'!$A:$A,0)),"past","past niet")),M14))</f>
-        <v>nog meten: waarschijnlijk (heeft weinig zadelpen nodig)</v>
+        <v>past</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="N14" s="5" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="O14" s="5" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="P14" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="Q14" s="6"/>
+        <v>132</v>
+      </c>
+      <c r="Q14" s="7"/>
     </row>
     <row r="15" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="C15" s="10" t="n">
         <v>10</v>
@@ -2251,7 +2292,7 @@
         <v>5.699</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="J15" s="5"/>
       <c r="K15" s="5" t="s">
@@ -2259,34 +2300,34 @@
       </c>
       <c r="L15" s="5" t="str">
         <f aca="false">IF(OR(J15="",K15=""),M15,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K15,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M15,IF(J15&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K15,'Mijn fiets'!$A:$A,0)),"past","past niet")),M15))</f>
-        <v>afhankelijk van ruimte zadel-band</v>
+        <v>waarschijnlijk: 22 cm zadelpen zichtbaar (ruimte zadel-band nog meten)</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="N15" s="5" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="P15" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="Q15" s="6"/>
+        <v>136</v>
+      </c>
+      <c r="Q15" s="7"/>
     </row>
     <row r="16" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="C16" s="10" t="n">
         <v>15</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="E16" s="10" t="n">
         <v>195</v>
@@ -2303,40 +2344,42 @@
         <v>1.4</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="J16" s="5"/>
+        <v>140</v>
+      </c>
+      <c r="J16" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="K16" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="L16" s="5" t="str">
         <f aca="false">IF(OR(J16="",K16=""),M16,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K16,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M16,IF(J16&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K16,'Mijn fiets'!$A:$A,0)),"past","past niet")),M16))</f>
-        <v>kort oprollen (≈ 30-35 cm) zodat de hoods vrij blijven</v>
+        <v>past</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="N16" s="5" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="O16" s="5" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="P16" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="Q16" s="6"/>
+        <v>143</v>
+      </c>
+      <c r="Q16" s="7"/>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="E17" s="10" t="n">
         <v>492</v>
@@ -2353,42 +2396,44 @@
         <v/>
       </c>
       <c r="I17" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="J17" s="5"/>
+        <v>146</v>
+      </c>
+      <c r="J17" s="10" t="n">
+        <v>40</v>
+      </c>
       <c r="K17" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="L17" s="5" t="str">
         <f aca="false">IF(OR(J17="",K17=""),M17,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K17,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M17,IF(J17&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K17,'Mijn fiets'!$A:$A,0)),"past","past niet")),M17))</f>
-        <v>40 cm breed op een 42 cm stuur: krap maar gangbaar</v>
+        <v>past niet</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="N17" s="5" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="O17" s="5" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="P17" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="Q17" s="6"/>
-    </row>
-    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>149</v>
+      </c>
+      <c r="Q17" s="7"/>
+    </row>
+    <row r="18" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="C18" s="10" t="n">
         <v>9</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="E18" s="10" t="n">
         <v>375</v>
@@ -2403,34 +2448,36 @@
         <v/>
       </c>
       <c r="I18" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="J18" s="5"/>
+        <v>152</v>
+      </c>
+      <c r="J18" s="10" t="n">
+        <v>40</v>
+      </c>
       <c r="K18" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="L18" s="5" t="str">
         <f aca="false">IF(OR(J18="",K18=""),M18,IFERROR(IF(INDEX('Mijn fiets'!$C:$C,MATCH(K18,'Mijn fiets'!$A:$A,0))="","nog meten: "&amp;M18,IF(J18&lt;=INDEX('Mijn fiets'!$C:$C,MATCH(K18,'Mijn fiets'!$A:$A,0)),"past","past niet")),M18))</f>
-        <v>de 9 L is de versie voor racesturen</v>
+        <v>past niet</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="N18" s="5" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="O18" s="5"/>
       <c r="P18" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="Q18" s="6"/>
+        <v>155</v>
+      </c>
+      <c r="Q18" s="7"/>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C19" s="10" t="n">
         <v>1</v>
@@ -2451,7 +2498,7 @@
         <v>24.99</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="J19" s="5"/>
       <c r="K19" s="5"/>
@@ -2460,31 +2507,31 @@
         <v>past (bandjes, geen boutjes nodig)</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="N19" s="5" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="O19" s="5" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="P19" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="Q19" s="6"/>
+        <v>162</v>
+      </c>
+      <c r="Q19" s="7"/>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="C20" s="10" t="n">
         <v>0.75</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="E20" s="10" t="n">
         <v>169</v>
@@ -2501,7 +2548,7 @@
         <v>30.6</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="J20" s="5"/>
       <c r="K20" s="5"/>
@@ -2510,25 +2557,25 @@
         <v>past (bandjes)</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="N20" s="5" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="O20" s="5" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="P20" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="Q20" s="6"/>
+        <v>168</v>
+      </c>
+      <c r="Q20" s="7"/>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="C21" s="10" t="n">
         <v>1</v>
@@ -2549,7 +2596,7 @@
         <v>26.95</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="J21" s="5"/>
       <c r="K21" s="5"/>
@@ -2558,25 +2605,25 @@
         <v>past</v>
       </c>
       <c r="M21" s="5" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="N21" s="5" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="O21" s="5" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="P21" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="Q21" s="6"/>
+        <v>174</v>
+      </c>
+      <c r="Q21" s="7"/>
     </row>
     <row r="22" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
@@ -2591,7 +2638,7 @@
         <v/>
       </c>
       <c r="I22" s="5" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="J22" s="5"/>
       <c r="K22" s="5"/>
@@ -2600,21 +2647,21 @@
         <v>past niet</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="N22" s="5" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="O22" s="5"/>
       <c r="P22" s="5"/>
-      <c r="Q22" s="6"/>
+      <c r="Q22" s="7"/>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
@@ -2629,7 +2676,7 @@
         <v/>
       </c>
       <c r="I23" s="5" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="J23" s="5"/>
       <c r="K23" s="5"/>
@@ -2638,21 +2685,21 @@
         <v>past niet</v>
       </c>
       <c r="M23" s="5" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="N23" s="5" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="O23" s="5"/>
       <c r="P23" s="5"/>
-      <c r="Q23" s="6"/>
+      <c r="Q23" s="7"/>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
@@ -2667,7 +2714,7 @@
         <v/>
       </c>
       <c r="I24" s="5" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="J24" s="5"/>
       <c r="K24" s="5"/>
@@ -2676,14 +2723,14 @@
         <v>past alleen zonder bidons</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="N24" s="5" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="O24" s="5"/>
       <c r="P24" s="5"/>
-      <c r="Q24" s="6"/>
+      <c r="Q24" s="7"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q24"/>
@@ -2751,27 +2798,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B2" s="15" t="n">
         <f aca="false">COUNTIFS(Uitrusting!$A:$A,A2,Uitrusting!$Q:$Q,"x")</f>
@@ -2796,7 +2843,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B3" s="15" t="n">
         <f aca="false">COUNTIFS(Uitrusting!$A:$A,A3,Uitrusting!$Q:$Q,"x")</f>
@@ -2821,7 +2868,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B4" s="15" t="n">
         <f aca="false">COUNTIFS(Uitrusting!$A:$A,A4,Uitrusting!$Q:$Q,"x")</f>
@@ -2846,7 +2893,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B5" s="15" t="n">
         <f aca="false">COUNTIFS(Uitrusting!$A:$A,A5,Uitrusting!$Q:$Q,"x")</f>
@@ -2871,7 +2918,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B6" s="15" t="n">
         <f aca="false">COUNTIFS(Uitrusting!$A:$A,A6,Uitrusting!$Q:$Q,"x")</f>
@@ -2896,7 +2943,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B7" s="18" t="n">
         <f aca="false">SUM(B2:B6)</f>
@@ -2921,7 +2968,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>